<commit_message>
Methodik + Testfälle Register Auswertung
</commit_message>
<xml_diff>
--- a/Testdaten/Testdaten von und für GPT-4/Register/Register_Account - ausgewertet.xlsx
+++ b/Testdaten/Testdaten von und für GPT-4/Register/Register_Account - ausgewertet.xlsx
@@ -1,20 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marvi\Desktop\Bachelor-Thesis\Testdaten\Testdaten von und für GPT-4\Register\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88358D21-37E0-4575-9F34-E181A92920D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="121">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -214,64 +233,104 @@
     <t>Validate Navigation Elements</t>
   </si>
   <si>
-    <t>Click on 'Register' button</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Check if 'Username', 'First Name', 'Last Name', 'E-Mail', 'Country', 'Password', and Captcha are present</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Click 'Register' without entering any data</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Fill all fields with valid data, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Use an already registered username, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Enter an incorrect email format (e.g., 'invalidemail@'), Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Fill all fields except one (Username, E-Mail, or Password), Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Enter username with 1 or more than 20 characters, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Enter first name with 1 or more than 32 characters, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Enter last name with 1 or more than 32 characters, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Use the same value for 'Username' and 'Password', Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Use special characters in 'Username', 'First Name', 'Last Name', 'E-Mail', Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Select wrong Captcha option, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Select correct Captcha option, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Use an email that is already registered, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Complete registration, Click 'Register', Check if email confirmation is received</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Complete registration with valid email but do not receive confirmation email, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Enter details, navigate back, then return to the form, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Verify if 'Register' button is disabled until form is filled correctly, Click 'Register'</t>
-  </si>
-  <si>
-    <t>Click on 'Register' button, Verify 'Features', 'Demo', 'Marketplace', 'Blog', 'Download', 'Resources', 'Login', and 'Register' links are present</t>
+    <t>1. Click on 'Register' button</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Check if 'Username', 'First Name', 'Last Name', 'E-Mail', 'Country', 'Password', and Captcha are present</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Click 'Register' without entering any data</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Fill all fields with valid data
+3. Click 'Register'
+4. User is redirected to confirmation page
+5. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Use an already registered username
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Enter an incorrect email format (e.g., 'invalidemail@')
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Fill all fields except one (Username, E-Mail, or Password)
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Enter username with 1 or more than 20 characters
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Enter first name with 1 or more than 32 characters
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Enter last name with 1 or more than 32 characters
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Use the same value for 'Username' and 'Password'
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Use special characters in 'Username', 'First Name', 'Last Name', 'E-Mail'
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Select wrong Captcha option
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Select correct Captcha option
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Use an email that is already registered
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Complete registration
+3. Click 'Register'
+4. User is redirected to confirmation page
+5. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Complete registration with valid email but do not receive confirmation email
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Enter details
+3. Navigate back, then return to the form
+4. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Verify if 'Register' button is disabled until form is filled correctly
+3. Click 'Register'</t>
+  </si>
+  <si>
+    <t>1. Click on 'Register' button
+2. Verify 'Features', 'Demo', 'Marketplace', 'Blog', 'Download', 'Resources', 'Login', and 'Register' links are present</t>
   </si>
   <si>
     <t>Registration form appears</t>
@@ -283,7 +342,7 @@
     <t>Error messages for all required fields</t>
   </si>
   <si>
-    <t>Registration successful, confirmation email sent</t>
+    <t>Welcome message appears, verification email is sent</t>
   </si>
   <si>
     <t>Error: 'Username is already registered'</t>
@@ -332,13 +391,101 @@
   </si>
   <si>
     <t>All navigation elements should be visible and clickable</t>
+  </si>
+  <si>
+    <t>Testfallstruktur eingehalten?</t>
+  </si>
+  <si>
+    <t>Factual Correctness</t>
+  </si>
+  <si>
+    <t>Abdeckung</t>
+  </si>
+  <si>
+    <t>Ja</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+TN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+TN = 1
+Button "Register" wird nicht gecheckt
+P = 0,5
+R = 0,5
+F1 = 0,5</t>
+  </si>
+  <si>
+    <t>TP = 2
+FP = 0
+TN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 5
+FP = 0
+TN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 3
+FP = 0
+TN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>TP = 4
+FP = 0
+TN = 0
+P = 1
+R = 1
+F1 = 1</t>
+  </si>
+  <si>
+    <t>Testfall Anzahl
+Pavankumar</t>
+  </si>
+  <si>
+    <t>Abdeckungsrate:</t>
+  </si>
+  <si>
+    <t>(17/27) * 100
+= 62,9%</t>
+  </si>
+  <si>
+    <t>TP = 2
+FP = 0
+TN = 1 Es wird nicht nach First Name und Last Name gecheckt
+P = 2/3
+R = 2/3
+F1 = 2/3</t>
+  </si>
+  <si>
+    <t>TP = 1
+FP = 0
+TN = 1, Es wird nicht geschaut ob auch "Opencart angezeigt wird", dieses ist jedoch auch in der Leiste
+P = 0,5
+R = 0,5
+F1 = 0,5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -355,12 +502,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -390,24 +549,53 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -445,7 +633,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -479,6 +667,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -513,9 +702,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -688,11 +878,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="33.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -711,408 +912,620 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="G1" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
+      <c r="G2" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="I2" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="3" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
+      <c r="G3" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="I3" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
+      <c r="G4" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="I4" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
+      <c r="G5" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I5" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="3" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
+      <c r="G6" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I6" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="3" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
+      <c r="G7" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I7" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="3" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
+      <c r="G8" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="I8" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="3" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
+      <c r="G9" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I9" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
+      <c r="G10" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I10" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C11" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="3" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
+      <c r="G11" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I11" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="C12" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
+      <c r="G12" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I12" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C13" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="C13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
+      <c r="G13" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I13" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="C14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="3" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
+      <c r="G14" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I14" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="C15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="3" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
+      <c r="G15" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I15" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C16" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="C16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="3" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
+      <c r="G16" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I16" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="C17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="3" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
+      <c r="G17" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I17" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="C18" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="3" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
+      <c r="G18" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I18" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C19" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="C19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" t="s">
+      <c r="G19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="I19" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C20" t="s">
-        <v>46</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="C20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
+      <c r="G20" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I20" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C21" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="3" t="s">
         <v>105</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I21" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I22" s="8">
+        <f>SUM(I2:I21)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="H23" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="I23" s="7">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="H24" t="s">
+        <v>117</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>